<commit_message>
Add donate-embed, quote blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 8
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-chris-evert-v1.report.xlsx
+++ b/tools/importer/reports/import-chris-evert-v1.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="870" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="480">
   <si>
     <t>_reportFile</t>
   </si>
@@ -68,6 +68,24 @@
   </si>
   <si>
     <t>https://www.ustafoundation.com/en/home.html</t>
+  </si>
+  <si>
+    <t>drafts/block-samples/cards-profile-bio.report.json</t>
+  </si>
+  <si>
+    <t>["spacer","cards-profile-bio","metadata"]</t>
+  </si>
+  <si>
+    <t>drafts/block-samples/cards-profile-bio</t>
+  </si>
+  <si>
+    <t>2026-10-01T23:35:40.509Z</t>
+  </si>
+  <si>
+    <t>Cards Profile Bio — Block Sample</t>
+  </si>
+  <si>
+    <t>https://www.ustafoundation.com/en/home/who-we-are/leadership-and-staff.html</t>
   </si>
   <si>
     <t>en/home/get-involved.report.json</t>
@@ -210,6 +228,24 @@
     <t>https://www.ustafoundation.com/en/home/get-involved/special-funds.html</t>
   </si>
   <si>
+    <t>en/home/get-involved/young-professional-initiative.report.json</t>
+  </si>
+  <si>
+    <t>["hero-text-up-tall","center-intro(future-of-giving)","columns(what-is-ypi,image-right)","spacer(yellow-strip)","columns(impact,image-left,yellow)","quote-image(labanowski)","spacer(yellow-strip)","columns(ways,image-left,yellow)","spacer(trailing-black-band)"]</t>
+  </si>
+  <si>
+    <t>en/home/get-involved/young-professional-initiative</t>
+  </si>
+  <si>
+    <t>2026-09-08T22:47:49.236Z</t>
+  </si>
+  <si>
+    <t>Young Professional Initiative</t>
+  </si>
+  <si>
+    <t>https://www.ustafoundation.com/en/home/get-involved/young-professional-initiative.html</t>
+  </si>
+  <si>
     <t>en/home/news/2023-njtl-essay-contest-winners.report.json</t>
   </si>
   <si>
@@ -911,7 +947,7 @@
     <t>en/home/news/robin-montgomery-wimbledon-debut</t>
   </si>
   <si>
-    <t>2026-09-07T17:13:17.395Z</t>
+    <t>2026-09-09T22:11:28.631Z</t>
   </si>
   <si>
     <t>Excellence Team alumna Robin Montgomery makes Wimbledon debut, earns first Grand Slam main-draw win</t>
@@ -929,7 +965,7 @@
     <t>en/home/news/six-student-athletes-awarded-first-grants-frances-tiafoe-fund</t>
   </si>
   <si>
-    <t>2026-09-07T17:13:23.320Z</t>
+    <t>2026-09-14T20:06:51.110Z</t>
   </si>
   <si>
     <t>Six student-athletes awarded first-ever grants from the Frances Tiafoe Fund</t>
@@ -1403,19 +1439,16 @@
     <t>Leadership &amp; Staff</t>
   </si>
   <si>
-    <t>https://www.ustafoundation.com/en/home/who-we-are/leadership-and-staff.html</t>
-  </si>
-  <si>
     <t>en/home/get-involved/special-funds/chris-evert-50th-anniversary.report.json</t>
   </si>
   <si>
-    <t>["default-content(heading,center)","columns(campaign,image-right)","split-even(quote+donate)","spacer(trailing-black-band)"]</t>
+    <t>["heading(h3)+columns(image-right) in center-intro,split-5-6","split-even(quote+donate)","spacer(trailing-black-band)"]</t>
   </si>
   <si>
     <t>en/home/get-involved/special-funds/chris-evert-50th-anniversary</t>
   </si>
   <si>
-    <t>2026-09-08T21:50:11.450Z</t>
+    <t>2026-10-02T02:27:22.165Z</t>
   </si>
   <si>
     <t>Chris Evert 50th anniversary</t>
@@ -1810,7 +1843,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="5" width="50" customWidth="1"/>
@@ -1903,39 +1936,39 @@
         <v>14</v>
       </c>
       <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" t="s">
         <v>22</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>24</v>
-      </c>
-      <c r="J3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" t="s">
         <v>26</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
         <v>27</v>
       </c>
-      <c r="C4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" t="s">
         <v>28</v>
-      </c>
-      <c r="F4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" t="s">
-        <v>22</v>
       </c>
       <c r="H4" t="s">
         <v>29</v>
@@ -1967,7 +2000,7 @@
         <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="H5" t="s">
         <v>35</v>
@@ -1984,159 +2017,159 @@
         <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>39</v>
+        <v>12</v>
       </c>
       <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
         <v>40</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>14</v>
+      </c>
+      <c r="G6" t="s">
+        <v>28</v>
+      </c>
+      <c r="H6" t="s">
         <v>41</v>
       </c>
-      <c r="F6" t="s">
+      <c r="I6" t="s">
         <v>42</v>
       </c>
-      <c r="G6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" t="s">
+      <c r="J6" t="s">
         <v>43</v>
-      </c>
-      <c r="I6" t="s">
-        <v>12</v>
-      </c>
-      <c r="J6" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
         <v>45</v>
       </c>
-      <c r="B7" t="s">
+      <c r="D7" t="s">
         <v>46</v>
-      </c>
-      <c r="C7" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
       </c>
       <c r="E7" t="s">
         <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G7" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I7" t="s">
-        <v>49</v>
+        <v>12</v>
       </c>
       <c r="J7" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" t="s">
+        <v>14</v>
+      </c>
+      <c r="G8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" t="s">
+        <v>54</v>
+      </c>
+      <c r="I8" t="s">
+        <v>55</v>
+      </c>
+      <c r="J8" t="s">
         <v>50</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" t="s">
-        <v>40</v>
-      </c>
-      <c r="E8" t="s">
-        <v>51</v>
-      </c>
-      <c r="F8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" t="s">
-        <v>52</v>
-      </c>
-      <c r="I8" t="s">
-        <v>12</v>
-      </c>
-      <c r="J8" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>12</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>45</v>
       </c>
       <c r="D9" t="s">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="E9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F9" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G9" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="H9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I9" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="J9" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" t="s">
+        <v>14</v>
+      </c>
+      <c r="G10" t="s">
+        <v>28</v>
+      </c>
+      <c r="H10" t="s">
+        <v>63</v>
+      </c>
+      <c r="I10" t="s">
+        <v>64</v>
+      </c>
+      <c r="J10" t="s">
         <v>59</v>
-      </c>
-      <c r="B10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>61</v>
-      </c>
-      <c r="F10" t="s">
-        <v>14</v>
-      </c>
-      <c r="G10" t="s">
-        <v>22</v>
-      </c>
-      <c r="H10" t="s">
-        <v>62</v>
-      </c>
-      <c r="I10" t="s">
-        <v>63</v>
-      </c>
-      <c r="J10" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -2159,71 +2192,71 @@
         <v>14</v>
       </c>
       <c r="G11" t="s">
+        <v>28</v>
+      </c>
+      <c r="H11" t="s">
         <v>68</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>69</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>70</v>
-      </c>
-      <c r="J11" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>71</v>
+      </c>
+      <c r="B12" t="s">
         <v>72</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
         <v>73</v>
       </c>
-      <c r="C12" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
+        <v>14</v>
+      </c>
+      <c r="G12" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" t="s">
         <v>74</v>
       </c>
-      <c r="F12" t="s">
-        <v>14</v>
-      </c>
-      <c r="G12" t="s">
-        <v>68</v>
-      </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>75</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>76</v>
-      </c>
-      <c r="J12" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B13" t="s">
         <v>78</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
         <v>79</v>
       </c>
-      <c r="C13" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-      <c r="E13" t="s">
-        <v>80</v>
-      </c>
       <c r="F13" t="s">
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H13" t="s">
         <v>81</v>
@@ -2255,7 +2288,7 @@
         <v>14</v>
       </c>
       <c r="G14" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H14" t="s">
         <v>87</v>
@@ -2287,7 +2320,7 @@
         <v>14</v>
       </c>
       <c r="G15" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H15" t="s">
         <v>93</v>
@@ -2319,7 +2352,7 @@
         <v>14</v>
       </c>
       <c r="G16" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H16" t="s">
         <v>99</v>
@@ -2351,7 +2384,7 @@
         <v>14</v>
       </c>
       <c r="G17" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H17" t="s">
         <v>105</v>
@@ -2368,7 +2401,7 @@
         <v>108</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>109</v>
       </c>
       <c r="C18" t="s">
         <v>12</v>
@@ -2377,30 +2410,30 @@
         <v>12</v>
       </c>
       <c r="E18" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F18" t="s">
         <v>14</v>
       </c>
       <c r="G18" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H18" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I18" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="J18" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B19" t="s">
-        <v>97</v>
+        <v>115</v>
       </c>
       <c r="C19" t="s">
         <v>12</v>
@@ -2409,30 +2442,30 @@
         <v>12</v>
       </c>
       <c r="E19" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="F19" t="s">
         <v>14</v>
       </c>
       <c r="G19" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H19" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I19" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="J19" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B20" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C20" t="s">
         <v>12</v>
@@ -2441,30 +2474,30 @@
         <v>12</v>
       </c>
       <c r="E20" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F20" t="s">
         <v>14</v>
       </c>
       <c r="G20" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H20" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="I20" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="J20" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B21" t="s">
-        <v>124</v>
+        <v>109</v>
       </c>
       <c r="C21" t="s">
         <v>12</v>
@@ -2473,30 +2506,30 @@
         <v>12</v>
       </c>
       <c r="E21" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F21" t="s">
         <v>14</v>
       </c>
       <c r="G21" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H21" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I21" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="J21" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B22" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C22" t="s">
         <v>12</v>
@@ -2505,30 +2538,30 @@
         <v>12</v>
       </c>
       <c r="E22" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F22" t="s">
         <v>14</v>
       </c>
       <c r="G22" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H22" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I22" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="J22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B23" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="C23" t="s">
         <v>12</v>
@@ -2537,62 +2570,62 @@
         <v>12</v>
       </c>
       <c r="E23" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="F23" t="s">
         <v>14</v>
       </c>
       <c r="G23" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H23" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="I23" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="J23" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B24" t="s">
-        <v>12</v>
+        <v>91</v>
       </c>
       <c r="C24" t="s">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="D24" t="s">
-        <v>141</v>
+        <v>12</v>
       </c>
       <c r="E24" t="s">
         <v>142</v>
       </c>
       <c r="F24" t="s">
-        <v>42</v>
+        <v>14</v>
       </c>
       <c r="G24" t="s">
-        <v>12</v>
+        <v>80</v>
       </c>
       <c r="H24" t="s">
         <v>143</v>
       </c>
       <c r="I24" t="s">
-        <v>12</v>
+        <v>144</v>
       </c>
       <c r="J24" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B25" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C25" t="s">
         <v>12</v>
@@ -2601,62 +2634,62 @@
         <v>12</v>
       </c>
       <c r="E25" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F25" t="s">
         <v>14</v>
       </c>
       <c r="G25" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H25" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I25" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="J25" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B26" t="s">
-        <v>103</v>
+        <v>12</v>
       </c>
       <c r="C26" t="s">
-        <v>12</v>
+        <v>152</v>
       </c>
       <c r="D26" t="s">
-        <v>12</v>
+        <v>153</v>
       </c>
       <c r="E26" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="F26" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="G26" t="s">
-        <v>68</v>
+        <v>12</v>
       </c>
       <c r="H26" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="I26" t="s">
-        <v>152</v>
+        <v>12</v>
       </c>
       <c r="J26" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B27" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C27" t="s">
         <v>12</v>
@@ -2665,30 +2698,30 @@
         <v>12</v>
       </c>
       <c r="E27" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F27" t="s">
         <v>14</v>
       </c>
       <c r="G27" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H27" t="s">
+        <v>159</v>
+      </c>
+      <c r="I27" t="s">
+        <v>160</v>
+      </c>
+      <c r="J27" t="s">
         <v>156</v>
-      </c>
-      <c r="I27" t="s">
-        <v>157</v>
-      </c>
-      <c r="J27" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B28" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C28" t="s">
         <v>12</v>
@@ -2697,30 +2730,30 @@
         <v>12</v>
       </c>
       <c r="E28" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F28" t="s">
         <v>14</v>
       </c>
       <c r="G28" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H28" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I28" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="J28" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B29" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="C29" t="s">
         <v>12</v>
@@ -2729,30 +2762,30 @@
         <v>12</v>
       </c>
       <c r="E29" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="F29" t="s">
         <v>14</v>
       </c>
       <c r="G29" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H29" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="I29" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="J29" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C30" t="s">
         <v>12</v>
@@ -2761,30 +2794,30 @@
         <v>12</v>
       </c>
       <c r="E30" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F30" t="s">
         <v>14</v>
       </c>
       <c r="G30" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H30" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="I30" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="J30" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B31" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C31" t="s">
         <v>12</v>
@@ -2793,30 +2826,30 @@
         <v>12</v>
       </c>
       <c r="E31" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F31" t="s">
         <v>14</v>
       </c>
       <c r="G31" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H31" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="I31" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J31" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B32" t="s">
-        <v>180</v>
+        <v>91</v>
       </c>
       <c r="C32" t="s">
         <v>12</v>
@@ -2825,30 +2858,30 @@
         <v>12</v>
       </c>
       <c r="E32" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F32" t="s">
         <v>14</v>
       </c>
       <c r="G32" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H32" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I32" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="J32" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B33" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C33" t="s">
         <v>12</v>
@@ -2857,30 +2890,30 @@
         <v>12</v>
       </c>
       <c r="E33" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F33" t="s">
         <v>14</v>
       </c>
       <c r="G33" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H33" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="I33" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="J33" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B34" t="s">
-        <v>103</v>
+        <v>192</v>
       </c>
       <c r="C34" t="s">
         <v>12</v>
@@ -2889,30 +2922,30 @@
         <v>12</v>
       </c>
       <c r="E34" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F34" t="s">
         <v>14</v>
       </c>
       <c r="G34" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H34" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="I34" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J34" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="B35" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C35" t="s">
         <v>12</v>
@@ -2921,30 +2954,30 @@
         <v>12</v>
       </c>
       <c r="E35" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F35" t="s">
         <v>14</v>
       </c>
       <c r="G35" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H35" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="I35" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="J35" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B36" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C36" t="s">
         <v>12</v>
@@ -2953,30 +2986,30 @@
         <v>12</v>
       </c>
       <c r="E36" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F36" t="s">
         <v>14</v>
       </c>
       <c r="G36" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H36" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="I36" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="J36" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="B37" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C37" t="s">
         <v>12</v>
@@ -2985,30 +3018,30 @@
         <v>12</v>
       </c>
       <c r="E37" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="F37" t="s">
         <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H37" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="I37" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="J37" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B38" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
         <v>12</v>
@@ -3017,30 +3050,30 @@
         <v>12</v>
       </c>
       <c r="E38" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F38" t="s">
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H38" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="I38" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="J38" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C39" t="s">
         <v>12</v>
@@ -3049,30 +3082,30 @@
         <v>12</v>
       </c>
       <c r="E39" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="F39" t="s">
         <v>14</v>
       </c>
       <c r="G39" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H39" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="I39" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="J39" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B40" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C40" t="s">
         <v>12</v>
@@ -3081,30 +3114,30 @@
         <v>12</v>
       </c>
       <c r="E40" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F40" t="s">
         <v>14</v>
       </c>
       <c r="G40" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H40" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="I40" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="J40" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="B41" t="s">
-        <v>226</v>
+        <v>91</v>
       </c>
       <c r="C41" t="s">
         <v>12</v>
@@ -3113,30 +3146,30 @@
         <v>12</v>
       </c>
       <c r="E41" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F41" t="s">
         <v>14</v>
       </c>
       <c r="G41" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H41" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I41" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="J41" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>115</v>
       </c>
       <c r="C42" t="s">
         <v>12</v>
@@ -3145,30 +3178,30 @@
         <v>12</v>
       </c>
       <c r="E42" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F42" t="s">
         <v>14</v>
       </c>
       <c r="G42" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H42" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="I42" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="J42" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B43" t="s">
-        <v>79</v>
+        <v>238</v>
       </c>
       <c r="C43" t="s">
         <v>12</v>
@@ -3177,30 +3210,30 @@
         <v>12</v>
       </c>
       <c r="E43" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="F43" t="s">
         <v>14</v>
       </c>
       <c r="G43" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H43" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="I43" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="J43" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="B44" t="s">
-        <v>103</v>
+        <v>91</v>
       </c>
       <c r="C44" t="s">
         <v>12</v>
@@ -3209,30 +3242,30 @@
         <v>12</v>
       </c>
       <c r="E44" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F44" t="s">
         <v>14</v>
       </c>
       <c r="G44" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H44" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="I44" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="J44" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B45" t="s">
-        <v>79</v>
+        <v>91</v>
       </c>
       <c r="C45" t="s">
         <v>12</v>
@@ -3241,30 +3274,30 @@
         <v>12</v>
       </c>
       <c r="E45" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="F45" t="s">
         <v>14</v>
       </c>
       <c r="G45" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H45" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="I45" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="J45" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B46" t="s">
-        <v>180</v>
+        <v>115</v>
       </c>
       <c r="C46" t="s">
         <v>12</v>
@@ -3273,30 +3306,30 @@
         <v>12</v>
       </c>
       <c r="E46" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F46" t="s">
         <v>14</v>
       </c>
       <c r="G46" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H46" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="I46" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="J46" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B47" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C47" t="s">
         <v>12</v>
@@ -3305,30 +3338,30 @@
         <v>12</v>
       </c>
       <c r="E47" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F47" t="s">
         <v>14</v>
       </c>
       <c r="G47" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H47" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="I47" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="J47" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="B48" t="s">
-        <v>124</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
         <v>12</v>
@@ -3337,30 +3370,30 @@
         <v>12</v>
       </c>
       <c r="E48" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F48" t="s">
         <v>14</v>
       </c>
       <c r="G48" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H48" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="I48" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="J48" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B49" t="s">
-        <v>267</v>
+        <v>109</v>
       </c>
       <c r="C49" t="s">
         <v>12</v>
@@ -3369,30 +3402,30 @@
         <v>12</v>
       </c>
       <c r="E49" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="F49" t="s">
         <v>14</v>
       </c>
       <c r="G49" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H49" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="I49" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J49" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B50" t="s">
-        <v>103</v>
+        <v>136</v>
       </c>
       <c r="C50" t="s">
         <v>12</v>
@@ -3401,30 +3434,30 @@
         <v>12</v>
       </c>
       <c r="E50" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F50" t="s">
         <v>14</v>
       </c>
       <c r="G50" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H50" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="I50" t="s">
-        <v>148</v>
+        <v>276</v>
       </c>
       <c r="J50" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="B51" t="s">
-        <v>103</v>
+        <v>279</v>
       </c>
       <c r="C51" t="s">
         <v>12</v>
@@ -3433,30 +3466,30 @@
         <v>12</v>
       </c>
       <c r="E51" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="F51" t="s">
         <v>14</v>
       </c>
       <c r="G51" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H51" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="I51" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="J51" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B52" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C52" t="s">
         <v>12</v>
@@ -3465,30 +3498,30 @@
         <v>12</v>
       </c>
       <c r="E52" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="F52" t="s">
         <v>14</v>
       </c>
       <c r="G52" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H52" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="I52" t="s">
-        <v>284</v>
+        <v>160</v>
       </c>
       <c r="J52" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B53" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C53" t="s">
         <v>12</v>
@@ -3497,30 +3530,30 @@
         <v>12</v>
       </c>
       <c r="E53" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F53" t="s">
         <v>14</v>
       </c>
       <c r="G53" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H53" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="I53" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="J53" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="B54" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C54" t="s">
         <v>12</v>
@@ -3529,30 +3562,30 @@
         <v>12</v>
       </c>
       <c r="E54" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="F54" t="s">
         <v>14</v>
       </c>
       <c r="G54" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H54" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="I54" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="J54" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="B55" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C55" t="s">
         <v>12</v>
@@ -3561,30 +3594,30 @@
         <v>12</v>
       </c>
       <c r="E55" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F55" t="s">
         <v>14</v>
       </c>
       <c r="G55" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H55" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="I55" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="J55" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="B56" t="s">
-        <v>302</v>
+        <v>115</v>
       </c>
       <c r="C56" t="s">
         <v>12</v>
@@ -3593,30 +3626,30 @@
         <v>12</v>
       </c>
       <c r="E56" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="F56" t="s">
         <v>14</v>
       </c>
       <c r="G56" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H56" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="I56" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="J56" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B57" t="s">
-        <v>103</v>
+        <v>192</v>
       </c>
       <c r="C57" t="s">
         <v>12</v>
@@ -3625,30 +3658,30 @@
         <v>12</v>
       </c>
       <c r="E57" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="F57" t="s">
         <v>14</v>
       </c>
       <c r="G57" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H57" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="I57" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="J57" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B58" t="s">
-        <v>73</v>
+        <v>314</v>
       </c>
       <c r="C58" t="s">
         <v>12</v>
@@ -3657,30 +3690,30 @@
         <v>12</v>
       </c>
       <c r="E58" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="F58" t="s">
         <v>14</v>
       </c>
       <c r="G58" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H58" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="I58" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="J58" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B59" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C59" t="s">
         <v>12</v>
@@ -3689,30 +3722,30 @@
         <v>12</v>
       </c>
       <c r="E59" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="F59" t="s">
         <v>14</v>
       </c>
       <c r="G59" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H59" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="I59" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="J59" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="B60" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C60" t="s">
         <v>12</v>
@@ -3721,30 +3754,30 @@
         <v>12</v>
       </c>
       <c r="E60" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F60" t="s">
         <v>14</v>
       </c>
       <c r="G60" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H60" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="I60" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="J60" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="B61" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="C61" t="s">
         <v>12</v>
@@ -3753,30 +3786,30 @@
         <v>12</v>
       </c>
       <c r="E61" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="F61" t="s">
         <v>14</v>
       </c>
       <c r="G61" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H61" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="I61" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="J61" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="B62" t="s">
-        <v>103</v>
+        <v>115</v>
       </c>
       <c r="C62" t="s">
         <v>12</v>
@@ -3785,30 +3818,30 @@
         <v>12</v>
       </c>
       <c r="E62" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="F62" t="s">
         <v>14</v>
       </c>
       <c r="G62" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H62" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="I62" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="J62" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="B63" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C63" t="s">
         <v>12</v>
@@ -3817,30 +3850,30 @@
         <v>12</v>
       </c>
       <c r="E63" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F63" t="s">
         <v>14</v>
       </c>
       <c r="G63" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H63" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="I63" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="J63" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="B64" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="C64" t="s">
         <v>12</v>
@@ -3849,30 +3882,30 @@
         <v>12</v>
       </c>
       <c r="E64" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="F64" t="s">
         <v>14</v>
       </c>
       <c r="G64" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H64" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="I64" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="J64" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="B65" t="s">
-        <v>348</v>
+        <v>115</v>
       </c>
       <c r="C65" t="s">
         <v>12</v>
@@ -3881,30 +3914,30 @@
         <v>12</v>
       </c>
       <c r="E65" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="F65" t="s">
         <v>14</v>
       </c>
       <c r="G65" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H65" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I65" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="J65" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B66" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="C66" t="s">
         <v>12</v>
@@ -3913,30 +3946,30 @@
         <v>12</v>
       </c>
       <c r="E66" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="F66" t="s">
         <v>14</v>
       </c>
       <c r="G66" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H66" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="I66" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="J66" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B67" t="s">
-        <v>97</v>
+        <v>360</v>
       </c>
       <c r="C67" t="s">
         <v>12</v>
@@ -3945,30 +3978,30 @@
         <v>12</v>
       </c>
       <c r="E67" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="F67" t="s">
         <v>14</v>
       </c>
       <c r="G67" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H67" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="I67" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="J67" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B68" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C68" t="s">
         <v>12</v>
@@ -3977,30 +4010,30 @@
         <v>12</v>
       </c>
       <c r="E68" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="F68" t="s">
         <v>14</v>
       </c>
       <c r="G68" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H68" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="I68" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="J68" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="B69" t="s">
-        <v>369</v>
+        <v>109</v>
       </c>
       <c r="C69" t="s">
         <v>12</v>
@@ -4009,30 +4042,30 @@
         <v>12</v>
       </c>
       <c r="E69" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="F69" t="s">
         <v>14</v>
       </c>
       <c r="G69" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H69" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="I69" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="J69" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B70" t="s">
-        <v>226</v>
+        <v>115</v>
       </c>
       <c r="C70" t="s">
         <v>12</v>
@@ -4041,30 +4074,30 @@
         <v>12</v>
       </c>
       <c r="E70" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="F70" t="s">
         <v>14</v>
       </c>
       <c r="G70" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H70" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="I70" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="J70" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B71" t="s">
-        <v>73</v>
+        <v>381</v>
       </c>
       <c r="C71" t="s">
         <v>12</v>
@@ -4073,30 +4106,30 @@
         <v>12</v>
       </c>
       <c r="E71" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="F71" t="s">
         <v>14</v>
       </c>
       <c r="G71" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H71" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="I71" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="J71" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="B72" t="s">
-        <v>73</v>
+        <v>238</v>
       </c>
       <c r="C72" t="s">
         <v>12</v>
@@ -4105,30 +4138,30 @@
         <v>12</v>
       </c>
       <c r="E72" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="F72" t="s">
         <v>14</v>
       </c>
       <c r="G72" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H72" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="I72" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="J72" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B73" t="s">
-        <v>302</v>
+        <v>85</v>
       </c>
       <c r="C73" t="s">
         <v>12</v>
@@ -4137,30 +4170,30 @@
         <v>12</v>
       </c>
       <c r="E73" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="F73" t="s">
         <v>14</v>
       </c>
       <c r="G73" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H73" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="I73" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="J73" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="B74" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C74" t="s">
         <v>12</v>
@@ -4169,30 +4202,30 @@
         <v>12</v>
       </c>
       <c r="E74" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="F74" t="s">
         <v>14</v>
       </c>
       <c r="G74" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H74" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="I74" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="J74" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="B75" t="s">
-        <v>103</v>
+        <v>314</v>
       </c>
       <c r="C75" t="s">
         <v>12</v>
@@ -4201,30 +4234,30 @@
         <v>12</v>
       </c>
       <c r="E75" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="F75" t="s">
         <v>14</v>
       </c>
       <c r="G75" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H75" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="I75" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="J75" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="B76" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="C76" t="s">
         <v>12</v>
@@ -4233,30 +4266,30 @@
         <v>12</v>
       </c>
       <c r="E76" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="F76" t="s">
         <v>14</v>
       </c>
       <c r="G76" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H76" t="s">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="I76" t="s">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="J76" t="s">
-        <v>408</v>
+        <v>410</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="B77" t="s">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="C77" t="s">
         <v>12</v>
@@ -4265,30 +4298,30 @@
         <v>12</v>
       </c>
       <c r="E77" t="s">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="F77" t="s">
         <v>14</v>
       </c>
       <c r="G77" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H77" t="s">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="I77" t="s">
-        <v>412</v>
+        <v>414</v>
       </c>
       <c r="J77" t="s">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="B78" t="s">
-        <v>226</v>
+        <v>85</v>
       </c>
       <c r="C78" t="s">
         <v>12</v>
@@ -4297,30 +4330,30 @@
         <v>12</v>
       </c>
       <c r="E78" t="s">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="F78" t="s">
         <v>14</v>
       </c>
       <c r="G78" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H78" t="s">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="I78" t="s">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="J78" t="s">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="B79" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C79" t="s">
         <v>12</v>
@@ -4329,30 +4362,30 @@
         <v>12</v>
       </c>
       <c r="E79" t="s">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="F79" t="s">
         <v>14</v>
       </c>
       <c r="G79" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H79" t="s">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="I79" t="s">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="J79" t="s">
-        <v>423</v>
+        <v>425</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="B80" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="C80" t="s">
         <v>12</v>
@@ -4361,30 +4394,30 @@
         <v>12</v>
       </c>
       <c r="E80" t="s">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="F80" t="s">
         <v>14</v>
       </c>
       <c r="G80" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H80" t="s">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="I80" t="s">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="J80" t="s">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B81" t="s">
-        <v>226</v>
+        <v>115</v>
       </c>
       <c r="C81" t="s">
         <v>12</v>
@@ -4393,30 +4426,30 @@
         <v>12</v>
       </c>
       <c r="E81" t="s">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="F81" t="s">
         <v>14</v>
       </c>
       <c r="G81" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H81" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="I81" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="J81" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="B82" t="s">
-        <v>124</v>
+        <v>238</v>
       </c>
       <c r="C82" t="s">
         <v>12</v>
@@ -4425,30 +4458,30 @@
         <v>12</v>
       </c>
       <c r="E82" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="F82" t="s">
         <v>14</v>
       </c>
       <c r="G82" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H82" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="I82" t="s">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="J82" t="s">
-        <v>438</v>
+        <v>440</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>439</v>
+        <v>441</v>
       </c>
       <c r="B83" t="s">
-        <v>79</v>
+        <v>238</v>
       </c>
       <c r="C83" t="s">
         <v>12</v>
@@ -4457,30 +4490,30 @@
         <v>12</v>
       </c>
       <c r="E83" t="s">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="F83" t="s">
         <v>14</v>
       </c>
       <c r="G83" t="s">
-        <v>68</v>
+        <v>80</v>
       </c>
       <c r="H83" t="s">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="I83" t="s">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="J83" t="s">
-        <v>443</v>
+        <v>445</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="B84" t="s">
-        <v>445</v>
+        <v>136</v>
       </c>
       <c r="C84" t="s">
         <v>12</v>
@@ -4489,30 +4522,30 @@
         <v>12</v>
       </c>
       <c r="E84" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="F84" t="s">
         <v>14</v>
       </c>
       <c r="G84" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="H84" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="I84" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="J84" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="B85" t="s">
-        <v>451</v>
+        <v>91</v>
       </c>
       <c r="C85" t="s">
         <v>12</v>
@@ -4527,7 +4560,7 @@
         <v>14</v>
       </c>
       <c r="G85" t="s">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="H85" t="s">
         <v>453</v>
@@ -4559,48 +4592,112 @@
         <v>14</v>
       </c>
       <c r="G86" t="s">
+        <v>28</v>
+      </c>
+      <c r="H86" t="s">
         <v>459</v>
       </c>
-      <c r="H86" t="s">
+      <c r="I86" t="s">
         <v>460</v>
       </c>
-      <c r="I86" t="s">
+      <c r="J86" t="s">
         <v>461</v>
-      </c>
-      <c r="J86" t="s">
-        <v>462</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>462</v>
+      </c>
+      <c r="B87" t="s">
         <v>463</v>
       </c>
-      <c r="B87" t="s">
+      <c r="C87" t="s">
+        <v>12</v>
+      </c>
+      <c r="D87" t="s">
+        <v>12</v>
+      </c>
+      <c r="E87" t="s">
         <v>464</v>
       </c>
-      <c r="C87" t="s">
-        <v>12</v>
-      </c>
-      <c r="D87" t="s">
-        <v>12</v>
-      </c>
-      <c r="E87" t="s">
+      <c r="F87" t="s">
+        <v>14</v>
+      </c>
+      <c r="G87" t="s">
+        <v>28</v>
+      </c>
+      <c r="H87" t="s">
         <v>465</v>
       </c>
-      <c r="F87" t="s">
-        <v>14</v>
-      </c>
-      <c r="G87" t="s">
-        <v>22</v>
-      </c>
-      <c r="H87" t="s">
+      <c r="I87" t="s">
         <v>466</v>
       </c>
-      <c r="I87" t="s">
+      <c r="J87" t="s">
         <v>467</v>
       </c>
-      <c r="J87" t="s">
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
         <v>468</v>
+      </c>
+      <c r="B88" t="s">
+        <v>469</v>
+      </c>
+      <c r="C88" t="s">
+        <v>12</v>
+      </c>
+      <c r="D88" t="s">
+        <v>12</v>
+      </c>
+      <c r="E88" t="s">
+        <v>470</v>
+      </c>
+      <c r="F88" t="s">
+        <v>14</v>
+      </c>
+      <c r="G88" t="s">
+        <v>471</v>
+      </c>
+      <c r="H88" t="s">
+        <v>472</v>
+      </c>
+      <c r="I88" t="s">
+        <v>473</v>
+      </c>
+      <c r="J88" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>474</v>
+      </c>
+      <c r="B89" t="s">
+        <v>475</v>
+      </c>
+      <c r="C89" t="s">
+        <v>12</v>
+      </c>
+      <c r="D89" t="s">
+        <v>12</v>
+      </c>
+      <c r="E89" t="s">
+        <v>476</v>
+      </c>
+      <c r="F89" t="s">
+        <v>14</v>
+      </c>
+      <c r="G89" t="s">
+        <v>28</v>
+      </c>
+      <c r="H89" t="s">
+        <v>477</v>
+      </c>
+      <c r="I89" t="s">
+        <v>478</v>
+      </c>
+      <c r="J89" t="s">
+        <v>479</v>
       </c>
     </row>
   </sheetData>

</xml_diff>